<commit_message>
feat(Packagers): combined get and post into a file, added condition of no excel file to read and write
</commit_message>
<xml_diff>
--- a/OR25-L-Interview Data.xlsx
+++ b/OR25-L-Interview Data.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Recruitment Responses" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Interview TimeTable" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Data Helper" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Data Helper And Info" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -664,7 +664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -675,6 +675,11 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>First time Startup</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>How to Add Dropdown</t>
         </is>
       </c>
@@ -686,6 +691,11 @@
         </is>
       </c>
       <c r="B2" t="inlineStr">
+        <is>
+          <t>Call getschedule for the year</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
         <is>
           <t>Go into data, click data validation, select list then select the area you want to get values from in the formula spot</t>
         </is>

</xml_diff>